<commit_message>
RENOVA CELL: anúncios e documentos usam https://renova-cell.vercel.app
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013VVvDZDB6MGd8kjnX4E42S
</commit_message>
<xml_diff>
--- a/projetos/renova-cell/06-campanhas/meta-ads/onda-0-montagem.xlsx
+++ b/projetos/renova-cell/06-campanhas/meta-ads/onda-0-montagem.xlsx
@@ -1218,7 +1218,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/quiz</t>
+          <t>https://renova-cell.vercel.app/quiz</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/offer</t>
+          <t>https://renova-cell.vercel.app/offer</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/offer</t>
+          <t>https://renova-cell.vercel.app/offer</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/offer</t>
+          <t>https://renova-cell.vercel.app/offer</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>https://SEU_DOMINIO/offer</t>
+          <t>https://renova-cell.vercel.app/offer</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">

</xml_diff>